<commit_message>
feat: resultados admin+operativo + carga con confirmacion + fix delate
</commit_message>
<xml_diff>
--- a/datos/Tablas Liquidación FedEx.xlsx
+++ b/datos/Tablas Liquidación FedEx.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A-Calidad\Documents\Liquidaciones_FedEx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\Liquidaciones_FedEx\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0415DFB0-7C39-410E-8925-7C27DBD4258E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D084C497-A376-4106-A4E3-FAF1EDAE73B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="4" xr2:uid="{CC85E23D-F8CE-4B4A-A179-DE172E72C50E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CC85E23D-F8CE-4B4A-A179-DE172E72C50E}"/>
   </bookViews>
   <sheets>
     <sheet name="Comercializadoras" sheetId="1" r:id="rId1"/>
     <sheet name="Etiquetas" sheetId="2" r:id="rId2"/>
-    <sheet name="Pasajeros" sheetId="3" r:id="rId3"/>
-    <sheet name="Art. 40" sheetId="4" r:id="rId4"/>
+    <sheet name="Art. 40" sheetId="4" r:id="rId3"/>
+    <sheet name="Pasajeros" sheetId="3" r:id="rId4"/>
     <sheet name="Fis" sheetId="5" r:id="rId5"/>
     <sheet name="DPA" sheetId="6" r:id="rId6"/>
     <sheet name="Hallazgos" sheetId="7" r:id="rId7"/>
@@ -2451,446 +2451,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF538DD5"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -3991,6 +3551,446 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF538DD5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -4005,88 +4005,88 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78AED981-1E62-42E8-AA5E-A754BFFE77D5}" name="Tabla1" displayName="Tabla1" ref="A1:D27" totalsRowShown="0" headerRowDxfId="99" dataDxfId="97" headerRowBorderDxfId="98" tableBorderDxfId="96" totalsRowBorderDxfId="95">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78AED981-1E62-42E8-AA5E-A754BFFE77D5}" name="Tabla1" displayName="Tabla1" ref="A1:D27" totalsRowShown="0" headerRowDxfId="82" dataDxfId="80" headerRowBorderDxfId="81" tableBorderDxfId="79" totalsRowBorderDxfId="78">
   <autoFilter ref="A1:D27" xr:uid="{78AED981-1E62-42E8-AA5E-A754BFFE77D5}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{C24D1D9A-B4E6-422F-84C2-3725823DF71A}" name="NO." dataDxfId="94"/>
-    <tableColumn id="2" xr3:uid="{ECB8970C-E3D4-4091-9C63-1818A3922A8B}" name="PAGO DE PEDIMENTO" dataDxfId="93" dataCellStyle="Normal 19"/>
-    <tableColumn id="3" xr3:uid="{94BD59D2-AB14-458F-BC2F-542E75392D92}" name="PEDIMENTO" dataDxfId="92" dataCellStyle="Normal 19"/>
-    <tableColumn id="4" xr3:uid="{3BEE2C23-EB13-4C84-A0C5-49E7FEDCB91B}" name="# GUÍA" dataDxfId="91" dataCellStyle="Normal 19"/>
+    <tableColumn id="1" xr3:uid="{C24D1D9A-B4E6-422F-84C2-3725823DF71A}" name="NO." dataDxfId="77"/>
+    <tableColumn id="2" xr3:uid="{ECB8970C-E3D4-4091-9C63-1818A3922A8B}" name="PAGO DE PEDIMENTO" dataDxfId="76" dataCellStyle="Normal 19"/>
+    <tableColumn id="3" xr3:uid="{94BD59D2-AB14-458F-BC2F-542E75392D92}" name="PEDIMENTO" dataDxfId="75" dataCellStyle="Normal 19"/>
+    <tableColumn id="4" xr3:uid="{3BEE2C23-EB13-4C84-A0C5-49E7FEDCB91B}" name="# GUÍA" dataDxfId="74" dataCellStyle="Normal 19"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{21AE80FF-942E-4FAE-B525-CE1C840A9551}" name="Tabla2" displayName="Tabla2" ref="A1:J12" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{21AE80FF-942E-4FAE-B525-CE1C840A9551}" name="Tabla2" displayName="Tabla2" ref="A1:J12" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72">
   <autoFilter ref="A1:J12" xr:uid="{21AE80FF-942E-4FAE-B525-CE1C840A9551}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{DB99CC35-4353-403C-8D10-4B57A2CBE4E0}" name="REFRENCIA" dataDxfId="88"/>
-    <tableColumn id="2" xr3:uid="{E2D8A000-8279-4301-84B8-92E7C4A33E7C}" name="NUMERO PEDIMENTO" dataDxfId="87"/>
-    <tableColumn id="3" xr3:uid="{5B4B39DD-5D3B-424A-82FA-A3D313BD2FE2}" name="TIPO" dataDxfId="86"/>
-    <tableColumn id="4" xr3:uid="{512C4DA2-1BC4-4FFB-9EC2-E7A901D1D607}" name="CAPTURISTA" dataDxfId="85"/>
-    <tableColumn id="5" xr3:uid="{32DCCD1D-9CCE-4DA5-B13F-65DB1B0BF87D}" name="CLAVE" dataDxfId="84"/>
-    <tableColumn id="6" xr3:uid="{42B7186E-5F8A-4CEB-88F5-D8757D624C5E}" name="CLIENTE" dataDxfId="83"/>
-    <tableColumn id="7" xr3:uid="{A11BDA10-01B3-43FC-8E41-179B0DE0568B}" name="F ENTRADA" dataDxfId="82"/>
-    <tableColumn id="8" xr3:uid="{629AD860-5BE4-4ED4-B86E-D00C9CF9BAC8}" name="F SALIDA" dataDxfId="81"/>
-    <tableColumn id="9" xr3:uid="{90B8CED3-9FE9-4334-BE5C-F15432FCE67D}" name="ETIQUETAS" dataDxfId="80"/>
-    <tableColumn id="10" xr3:uid="{008B4649-65AC-43BB-8240-FBE5807647F9}" name="CONS" dataDxfId="79"/>
+    <tableColumn id="1" xr3:uid="{DB99CC35-4353-403C-8D10-4B57A2CBE4E0}" name="REFRENCIA" dataDxfId="71"/>
+    <tableColumn id="2" xr3:uid="{E2D8A000-8279-4301-84B8-92E7C4A33E7C}" name="NUMERO PEDIMENTO" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{5B4B39DD-5D3B-424A-82FA-A3D313BD2FE2}" name="TIPO" dataDxfId="69"/>
+    <tableColumn id="4" xr3:uid="{512C4DA2-1BC4-4FFB-9EC2-E7A901D1D607}" name="CAPTURISTA" dataDxfId="68"/>
+    <tableColumn id="5" xr3:uid="{32DCCD1D-9CCE-4DA5-B13F-65DB1B0BF87D}" name="CLAVE" dataDxfId="67"/>
+    <tableColumn id="6" xr3:uid="{42B7186E-5F8A-4CEB-88F5-D8757D624C5E}" name="CLIENTE" dataDxfId="66"/>
+    <tableColumn id="7" xr3:uid="{A11BDA10-01B3-43FC-8E41-179B0DE0568B}" name="F ENTRADA" dataDxfId="65"/>
+    <tableColumn id="8" xr3:uid="{629AD860-5BE4-4ED4-B86E-D00C9CF9BAC8}" name="F SALIDA" dataDxfId="64"/>
+    <tableColumn id="9" xr3:uid="{90B8CED3-9FE9-4334-BE5C-F15432FCE67D}" name="ETIQUETAS" dataDxfId="63"/>
+    <tableColumn id="10" xr3:uid="{008B4649-65AC-43BB-8240-FBE5807647F9}" name="CONS" dataDxfId="62"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{687C2BDD-4A35-4FC6-A19F-90484B3C76F1}" name="Tabla3" displayName="Tabla3" ref="A1:J3" totalsRowShown="0" headerRowDxfId="78" dataDxfId="76" headerRowBorderDxfId="77" tableBorderDxfId="75" totalsRowBorderDxfId="74">
-  <autoFilter ref="A1:J3" xr:uid="{687C2BDD-4A35-4FC6-A19F-90484B3C76F1}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{335BF007-CEB5-4280-8F97-8DD601B8695B}" name="DESTINO" dataDxfId="73"/>
-    <tableColumn id="2" xr3:uid="{7EA8B444-49D6-41F5-A677-38A99338782F}" name="REASON CODE" dataDxfId="72"/>
-    <tableColumn id="3" xr3:uid="{5EC8B07E-5464-4236-9C08-F42BF6CE47B4}" name="No DE GUIA" dataDxfId="71"/>
-    <tableColumn id="4" xr3:uid="{EA287CE7-4E2E-4BDC-A970-DB5F7F20713D}" name="FECHA DE ENTRADA" dataDxfId="70"/>
-    <tableColumn id="5" xr3:uid="{9597653A-F74F-41D3-8461-A79E802DFAA5}" name="CLIENTE" dataDxfId="69"/>
-    <tableColumn id="6" xr3:uid="{A1BFC91E-34D3-4EE0-BA46-18DECA67703A}" name="DESCRIPCION DE LA MERCANCIA" dataDxfId="68"/>
-    <tableColumn id="7" xr3:uid="{D7DCC342-E3C3-482F-BBF3-415D1AA95C6B}" name="INFORMACION DE CONTACTO" dataDxfId="67" dataCellStyle="Hipervínculo"/>
-    <tableColumn id="8" xr3:uid="{02B3DF24-9385-49BB-A030-DF22EEA34CBA}" name="FECHA DE LIBERACION DE ADUANA" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{C8BCFF0C-D7C9-4851-BBC9-986134F017E8}" name="EJECUTIVO CS A CARGO" dataDxfId="65"/>
-    <tableColumn id="10" xr3:uid="{F187905F-EB4D-4103-8362-3768FAEA4F5F}" name="MES DE LIBERACION " dataDxfId="64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B559062B-6D0C-42A1-B4AC-05CEFC522192}" name="Tabla4" displayName="Tabla4" ref="A1:F9" totalsRowShown="0" headerRowDxfId="46" dataDxfId="44" headerRowBorderDxfId="45" tableBorderDxfId="43">
+  <autoFilter ref="A1:F9" xr:uid="{B559062B-6D0C-42A1-B4AC-05CEFC522192}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{5624A351-D5D9-44DF-A528-A8E3D5970EAE}" name="FECHA/PAGO" dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{2F3719B1-5615-4C27-8CC6-4D9C47A994FF}" name="OPERACIÓN" dataDxfId="41"/>
+    <tableColumn id="3" xr3:uid="{6E303380-C2B2-40A5-9443-3648BD4FC80E}" name="SERVICIO" dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{9191AA75-8F93-4A18-AC0D-CB69E1653FD2}" name="IMPORTE" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{F47EACBD-748B-40B3-BE39-7B034E4C20CA}" name="FECHA DEL SERVICIO" dataDxfId="38"/>
+    <tableColumn id="6" xr3:uid="{FA32F772-DE5A-4D17-A99F-A92A2B2854D4}" name="CLIENTE" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B559062B-6D0C-42A1-B4AC-05CEFC522192}" name="Tabla4" displayName="Tabla4" ref="A1:F9" totalsRowShown="0" headerRowDxfId="63" dataDxfId="61" headerRowBorderDxfId="62" tableBorderDxfId="60">
-  <autoFilter ref="A1:F9" xr:uid="{B559062B-6D0C-42A1-B4AC-05CEFC522192}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{5624A351-D5D9-44DF-A528-A8E3D5970EAE}" name="FECHA/PAGO" dataDxfId="59"/>
-    <tableColumn id="2" xr3:uid="{2F3719B1-5615-4C27-8CC6-4D9C47A994FF}" name="OPERACIÓN" dataDxfId="58"/>
-    <tableColumn id="3" xr3:uid="{6E303380-C2B2-40A5-9443-3648BD4FC80E}" name="SERVICIO" dataDxfId="57"/>
-    <tableColumn id="4" xr3:uid="{9191AA75-8F93-4A18-AC0D-CB69E1653FD2}" name="IMPORTE" dataDxfId="56"/>
-    <tableColumn id="5" xr3:uid="{F47EACBD-748B-40B3-BE39-7B034E4C20CA}" name="FECHA DEL SERVICIO" dataDxfId="55"/>
-    <tableColumn id="6" xr3:uid="{FA32F772-DE5A-4D17-A99F-A92A2B2854D4}" name="CLIENTE" dataDxfId="54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{687C2BDD-4A35-4FC6-A19F-90484B3C76F1}" name="Tabla3" displayName="Tabla3" ref="A1:J3" totalsRowShown="0" headerRowDxfId="61" dataDxfId="59" headerRowBorderDxfId="60" tableBorderDxfId="58" totalsRowBorderDxfId="57">
+  <autoFilter ref="A1:J3" xr:uid="{687C2BDD-4A35-4FC6-A19F-90484B3C76F1}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{335BF007-CEB5-4280-8F97-8DD601B8695B}" name="DESTINO" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{7EA8B444-49D6-41F5-A677-38A99338782F}" name="REASON CODE" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{5EC8B07E-5464-4236-9C08-F42BF6CE47B4}" name="No DE GUIA" dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{EA287CE7-4E2E-4BDC-A970-DB5F7F20713D}" name="FECHA DE ENTRADA" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{9597653A-F74F-41D3-8461-A79E802DFAA5}" name="CLIENTE" dataDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{A1BFC91E-34D3-4EE0-BA46-18DECA67703A}" name="DESCRIPCION DE LA MERCANCIA" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{D7DCC342-E3C3-482F-BBF3-415D1AA95C6B}" name="INFORMACION DE CONTACTO" dataDxfId="50" dataCellStyle="Hipervínculo"/>
+    <tableColumn id="8" xr3:uid="{02B3DF24-9385-49BB-A030-DF22EEA34CBA}" name="FECHA DE LIBERACION DE ADUANA" dataDxfId="49"/>
+    <tableColumn id="9" xr3:uid="{C8BCFF0C-D7C9-4851-BBC9-986134F017E8}" name="EJECUTIVO CS A CARGO" dataDxfId="48"/>
+    <tableColumn id="10" xr3:uid="{F187905F-EB4D-4103-8362-3768FAEA4F5F}" name="MES DE LIBERACION " dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{293532C3-253F-4DCE-B5CF-5D007B67D2B4}" name="Tabla5" displayName="Tabla5" ref="A1:M107" totalsRowShown="0" headerRowDxfId="53" dataDxfId="51" headerRowBorderDxfId="52" tableBorderDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{293532C3-253F-4DCE-B5CF-5D007B67D2B4}" name="Tabla5" displayName="Tabla5" ref="A1:M107" totalsRowShown="0" headerRowDxfId="99" dataDxfId="97" headerRowBorderDxfId="98" tableBorderDxfId="96">
   <autoFilter ref="A1:M107" xr:uid="{293532C3-253F-4DCE-B5CF-5D007B67D2B4}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{455EEA60-DB54-4736-BA6D-8CD6E97C1637}" name="REFRENCIA" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{2CB2FA5E-8D42-4E90-B197-F8AC765C7479}" name="NUMERO PEDIMENTO" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{232DC06C-894C-4768-BB27-00CDBA43B46F}" name="GUÍAS" dataDxfId="47"/>
-    <tableColumn id="4" xr3:uid="{7F8CE19D-E105-4E9B-9F78-ECF9DE6A867A}" name="TIPO" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{76EA06AE-49BA-4740-B535-2F604DD41ECA}" name="CAPTURISTA" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{75425006-1148-4E20-A8EE-19C78CB1B051}" name="CLAVE" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{7977EC44-C09D-455A-9F43-FD6DFFC8488B}" name="CLIENTE" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{3996587F-280A-4A14-9EC5-D371D45DD6B5}" name="F ENTRADA" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{C8EF7CFD-F57C-4CE7-A45A-881134C5AF85}" name="F SALIDA" dataDxfId="41"/>
-    <tableColumn id="10" xr3:uid="{63202B32-0884-4C97-8858-234316C50C91}" name="GUIAS2" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{12035D57-FE35-4802-A301-1D918561A9DA}" name="BULTOS" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{931749B6-98A0-4E21-942E-E47BF3D08DE3}" name="T OP" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{71CE017B-73FE-4D87-9BEB-8B6B1EC1D7F8}" name="GUÍAS ¨FIS" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{455EEA60-DB54-4736-BA6D-8CD6E97C1637}" name="REFRENCIA" dataDxfId="95"/>
+    <tableColumn id="2" xr3:uid="{2CB2FA5E-8D42-4E90-B197-F8AC765C7479}" name="NUMERO PEDIMENTO" dataDxfId="94"/>
+    <tableColumn id="3" xr3:uid="{232DC06C-894C-4768-BB27-00CDBA43B46F}" name="GUÍAS" dataDxfId="93"/>
+    <tableColumn id="4" xr3:uid="{7F8CE19D-E105-4E9B-9F78-ECF9DE6A867A}" name="TIPO" dataDxfId="92"/>
+    <tableColumn id="5" xr3:uid="{76EA06AE-49BA-4740-B535-2F604DD41ECA}" name="CAPTURISTA" dataDxfId="91"/>
+    <tableColumn id="6" xr3:uid="{75425006-1148-4E20-A8EE-19C78CB1B051}" name="CLAVE" dataDxfId="90"/>
+    <tableColumn id="7" xr3:uid="{7977EC44-C09D-455A-9F43-FD6DFFC8488B}" name="CLIENTE" dataDxfId="89"/>
+    <tableColumn id="8" xr3:uid="{3996587F-280A-4A14-9EC5-D371D45DD6B5}" name="F ENTRADA" dataDxfId="88"/>
+    <tableColumn id="9" xr3:uid="{C8EF7CFD-F57C-4CE7-A45A-881134C5AF85}" name="F SALIDA" dataDxfId="87"/>
+    <tableColumn id="10" xr3:uid="{63202B32-0884-4C97-8858-234316C50C91}" name="GUIAS2" dataDxfId="86"/>
+    <tableColumn id="11" xr3:uid="{12035D57-FE35-4802-A301-1D918561A9DA}" name="BULTOS" dataDxfId="85"/>
+    <tableColumn id="12" xr3:uid="{931749B6-98A0-4E21-942E-E47BF3D08DE3}" name="T OP" dataDxfId="84"/>
+    <tableColumn id="13" xr3:uid="{71CE017B-73FE-4D87-9BEB-8B6B1EC1D7F8}" name="GUÍAS ¨FIS" dataDxfId="83"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5244,6 +5244,200 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C6F962-8D0F-41DA-86C5-9BAC1715DC0D}">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A2" s="13">
+        <v>46142</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="C2" s="12">
+        <v>1</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E2" s="13">
+        <v>46147</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A3" s="13">
+        <v>46142</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="C3" s="12">
+        <v>1</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E3" s="13">
+        <v>46147</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A4" s="13">
+        <v>46142</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="C4" s="12">
+        <v>1</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E4" s="13">
+        <v>46147</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A5" s="13">
+        <v>46142</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="C5" s="12">
+        <v>1</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E5" s="13">
+        <v>46147</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A6" s="13">
+        <v>46142</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="C6" s="12">
+        <v>1</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E6" s="13">
+        <v>46147</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A7" s="13">
+        <v>46142</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="C7" s="12">
+        <v>1</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E7" s="13">
+        <v>46147</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A8" s="13">
+        <v>46199</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="C8" s="12">
+        <v>1</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E8" s="13">
+        <v>46199</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="28">
+        <f>SUM(C2:C8)</f>
+        <v>7</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EA2C1E6-8490-46ED-81E1-818F201A07A6}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -5364,200 +5558,6 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId3"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C6F962-8D0F-41DA-86C5-9BAC1715DC0D}">
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.453125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
-      <c r="A2" s="13">
-        <v>46142</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>268</v>
-      </c>
-      <c r="C2" s="12">
-        <v>1</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="E2" s="13">
-        <v>46147</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
-      <c r="A3" s="13">
-        <v>46142</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>271</v>
-      </c>
-      <c r="C3" s="12">
-        <v>1</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="E3" s="13">
-        <v>46147</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
-      <c r="A4" s="13">
-        <v>46142</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>271</v>
-      </c>
-      <c r="C4" s="12">
-        <v>1</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="E4" s="13">
-        <v>46147</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
-      <c r="A5" s="13">
-        <v>46142</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>271</v>
-      </c>
-      <c r="C5" s="12">
-        <v>1</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="E5" s="13">
-        <v>46147</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
-      <c r="A6" s="13">
-        <v>46142</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>271</v>
-      </c>
-      <c r="C6" s="12">
-        <v>1</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="E6" s="13">
-        <v>46147</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
-      <c r="A7" s="13">
-        <v>46142</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>271</v>
-      </c>
-      <c r="C7" s="12">
-        <v>1</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="E7" s="13">
-        <v>46147</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
-      <c r="A8" s="13">
-        <v>46199</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>268</v>
-      </c>
-      <c r="C8" s="12">
-        <v>1</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="E8" s="13">
-        <v>46199</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="7" customFormat="1" ht="12" x14ac:dyDescent="0.3">
-      <c r="A9" s="17"/>
-      <c r="B9" s="17"/>
-      <c r="C9" s="28">
-        <f>SUM(C2:C8)</f>
-        <v>7</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>276</v>
-      </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>